<commit_message>
Fix: filas de cafe corregidas, pipeline completo sin salteos
</commit_message>
<xml_diff>
--- a/data/manual/research_template_1.xlsx
+++ b/data/manual/research_template_1.xlsx
@@ -13,23 +13,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="144">
   <si>
     <t>LatamPulse — Template de Research Manual</t>
   </si>
   <si>
+    <t>Checklist — 13 items x 4 países = 52 precios a investigar. Tildá acá a medida que cargás cada uno en la hoja 'Research'.</t>
+  </si>
+  <si>
+    <t>Para qué sirve este archivo</t>
+  </si>
+  <si>
     <t>country</t>
   </si>
   <si>
-    <t>Checklist — 13 items x 4 países = 52 precios a investigar. Tildá acá a medida que cargás cada uno en la hoja 'Research'.</t>
-  </si>
-  <si>
     <t>✓</t>
   </si>
   <si>
-    <t>Para qué sirve este archivo</t>
-  </si>
-  <si>
     <t>category</t>
   </si>
   <si>
@@ -45,24 +45,27 @@
     <t>currency</t>
   </si>
   <si>
+    <t>date_captured</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
     <t>item</t>
   </si>
   <si>
-    <t>date_captured</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>confidence</t>
-  </si>
-  <si>
     <t>captured_by</t>
   </si>
   <si>
+    <t>AR</t>
+  </si>
+  <si>
     <t>Las fuentes oficiales (INDEC, IBGE, INE, DANE) no publican precios de items como Netflix, cine, cerveza en bar o Uber. Este template es donde cargás esos precios investigados a mano, con fecha y fuente — así el dato entra al pipeline con confidence = 'manual_research' y queda 100% trazable.</t>
   </si>
   <si>
@@ -72,84 +75,81 @@
     <t>1. Andá a la hoja 'Research' (la pestaña de al lado).</t>
   </si>
   <si>
-    <t>AR</t>
-  </si>
-  <si>
     <t>2. La primera fila de datos (resaltada en amarillo) es un EJEMPLO — mostrá el formato esperado, no la borres, usala de referencia y agregá tus filas debajo.</t>
   </si>
   <si>
     <t>3. Completá SOLO las columnas con fondo verde. El resto (usd_nominal, usd_ppp) se calcula después en transform.py — dejalas vacías.</t>
   </si>
   <si>
+    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
+  </si>
+  <si>
+    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
+  </si>
+  <si>
+    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
+  </si>
+  <si>
+    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
+  </si>
+  <si>
+    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
+  </si>
+  <si>
     <t>entretenimiento</t>
   </si>
   <si>
     <t>Netflix Estándar (mensual)</t>
   </si>
   <si>
+    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
+  </si>
+  <si>
     <t>suscripcion_mensual</t>
   </si>
   <si>
-    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
-  </si>
-  <si>
     <t>ARS</t>
   </si>
   <si>
-    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
-  </si>
-  <si>
-    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
+    <t>netflix.com/ar (rango oficial $8.999-$19.999) + fuentes secundarias feb-jul 2026</t>
+  </si>
+  <si>
+    <t>Precio corregido — el valor original cargado ($7.999) estaba por debajo incluso del plan más barato del rango oficial actual, probablemente desactualizado</t>
+  </si>
+  <si>
+    <t>manual_research</t>
+  </si>
+  <si>
+    <t>Juani</t>
+  </si>
+  <si>
+    <t>UY</t>
+  </si>
+  <si>
+    <t>Entrada de cine (1 persona, horario normal)</t>
+  </si>
+  <si>
+    <t>unidad</t>
+  </si>
+  <si>
+    <t>UYU</t>
+  </si>
+  <si>
+    <t>lifecinemas.com.uy/candy</t>
   </si>
   <si>
     <t>Spotify Individual (mensual)</t>
   </si>
   <si>
-    <t>netflix.com/ar (rango oficial $8.999-$19.999) + fuentes secundarias feb-jul 2026</t>
-  </si>
-  <si>
-    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
-  </si>
-  <si>
-    <t>Precio corregido — el valor original cargado ($7.999) estaba por debajo incluso del plan más barato del rango oficial actual, probablemente desactualizado</t>
-  </si>
-  <si>
-    <t>Entrada de cine (1 persona, horario normal)</t>
-  </si>
-  <si>
-    <t>unidad</t>
-  </si>
-  <si>
-    <t>manual_research</t>
-  </si>
-  <si>
-    <t>Juani</t>
-  </si>
-  <si>
     <t>Menú/plato principal, restaurante gama media (1 persona)</t>
   </si>
   <si>
-    <t>UY</t>
-  </si>
-  <si>
-    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
-  </si>
-  <si>
     <t>Cerveza nacional 0.5L, en bar/restaurante</t>
   </si>
   <si>
-    <t>UYU</t>
-  </si>
-  <si>
     <t>Café con leche/cortado, en cafetería</t>
   </si>
   <si>
-    <t>lifecinemas.com.uy/candy</t>
-  </si>
-  <si>
-    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
-  </si>
-  <si>
     <t>Gimnasio, membresía mensual</t>
   </si>
   <si>
@@ -180,18 +180,18 @@
     <t>Alquiler 2 ambientes, zona no céntrica (mensual)</t>
   </si>
   <si>
+    <t>Precio de lista sin promo, verificado en el sitio oficial</t>
+  </si>
+  <si>
     <t>salud</t>
   </si>
   <si>
+    <t>BR</t>
+  </si>
+  <si>
     <t>Prepaga/plan de salud privado, plan básico individual (mensual)</t>
   </si>
   <si>
-    <t>Precio de lista sin promo, verificado en el sitio oficial</t>
-  </si>
-  <si>
-    <t>BR</t>
-  </si>
-  <si>
     <t>BRL</t>
   </si>
   <si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>Precio promedio real de encuesta, no un rango estimado</t>
+  </si>
+  <si>
+    <t>1.5</t>
   </si>
   <si>
     <t>USD</t>
@@ -448,9 +451,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="d.m"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -466,14 +468,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <b/>
       <sz val="11.0"/>
       <color rgb="FF1F4E78"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -494,13 +496,13 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <i/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <sz val="10.0"/>
       <color theme="1"/>
@@ -605,10 +607,10 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -622,22 +624,22 @@
     <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -648,7 +650,7 @@
     <xf borderId="1" fillId="5" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="5" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -892,72 +894,72 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3"/>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" ht="18.0" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" ht="96.75" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>16</v>
+      <c r="A4" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3"/>
+      <c r="A5" s="2"/>
     </row>
     <row r="6" ht="18.0" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" ht="18.0" customHeight="1">
-      <c r="A7" s="3" t="s">
-        <v>18</v>
+      <c r="A7" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" ht="51.75" customHeight="1">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="42.75" customHeight="1">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" ht="64.5" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" ht="39.75" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" ht="70.5" customHeight="1">
+      <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" ht="64.5" customHeight="1">
-      <c r="A11" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" ht="39.75" customHeight="1">
-      <c r="A12" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" ht="70.5" customHeight="1">
-      <c r="A13" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="3"/>
+      <c r="A14" s="2"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" ht="91.5" customHeight="1">
-      <c r="A16" s="3" t="s">
-        <v>44</v>
+      <c r="A16" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1971,7 +1973,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>5</v>
@@ -1989,173 +1991,173 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="10">
+      <c r="A2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="8">
         <v>14999.0</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="14">
+      <c r="F2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="12">
         <v>46243.0</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" s="10" t="s">
+      <c r="H2" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="I2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="10" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="s">
+      <c r="B3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="8">
+        <v>570.0</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="12">
+        <v>46239.0</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="10">
-        <v>570.0</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="14">
-        <v>46239.0</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="10" t="s">
+      <c r="K3" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="8">
         <v>7.0</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="14">
+      <c r="G4" s="12">
         <v>46237.0</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="10" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="A5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="8">
+        <v>17900.0</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="12">
+        <v>46243.0</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="10">
-        <v>17900.0</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="14">
-        <v>46243.0</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="I5" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" s="10" t="s">
+      <c r="K5" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E6" s="16">
         <v>44.0</v>
@@ -2173,10 +2175,10 @@
         <v>65</v>
       </c>
       <c r="J6" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K6" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -2184,13 +2186,13 @@
         <v>66</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E7" s="16">
         <v>21250.0</v>
@@ -2208,30 +2210,30 @@
         <v>68</v>
       </c>
       <c r="J7" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E8" s="16">
         <v>22500.0</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G8" s="17">
         <v>46243.0</v>
@@ -2243,24 +2245,24 @@
         <v>69</v>
       </c>
       <c r="J8" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K8" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E9" s="16">
         <v>60.0</v>
@@ -2278,30 +2280,30 @@
         <v>71</v>
       </c>
       <c r="J9" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K9" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>34</v>
       </c>
       <c r="E10" s="16">
         <v>1005.0</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G10" s="17">
         <v>46243.0</v>
@@ -2313,10 +2315,10 @@
         <v>72</v>
       </c>
       <c r="J10" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K10" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -2324,13 +2326,13 @@
         <v>66</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E11" s="16">
         <v>45000.0</v>
@@ -2348,30 +2350,30 @@
         <v>73</v>
       </c>
       <c r="J11" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K11" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K11" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E12" s="16">
         <v>3336.0</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G12" s="17">
         <v>46243.0</v>
@@ -2383,65 +2385,65 @@
         <v>75</v>
       </c>
       <c r="J12" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K12" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K12" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="18">
-        <v>46143.0</v>
+        <v>38</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>76</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G13" s="17">
         <v>46243.0</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J13" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K13" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>34</v>
       </c>
       <c r="E14" s="16">
         <v>200.0</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G14" s="17">
         <v>46243.0</v>
@@ -2450,13 +2452,13 @@
         <v>64</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J14" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K14" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K14" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="15">
@@ -2464,54 +2466,54 @@
         <v>66</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="18">
-        <v>46143.0</v>
+        <v>38</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>76</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G15" s="17">
         <v>46243.0</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J15" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K15" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K15" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E16" s="16">
         <v>45000.0</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G16" s="17">
         <v>46243.0</v>
@@ -2520,27 +2522,27 @@
         <v>64</v>
       </c>
       <c r="I16" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J16" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K16" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E17" s="16">
         <v>115.0</v>
@@ -2555,48 +2557,48 @@
         <v>64</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J17" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K17" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E18" s="16">
         <v>1590.0</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G18" s="17">
         <v>46243.0</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J18" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K18" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="19">
@@ -2604,13 +2606,13 @@
         <v>66</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E19" s="16">
         <v>150000.0</v>
@@ -2625,18 +2627,18 @@
         <v>64</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J19" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K19" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B20" s="16" t="s">
         <v>46</v>
@@ -2645,13 +2647,13 @@
         <v>47</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E20" s="16">
         <v>5500.0</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G20" s="17">
         <v>46243.0</v>
@@ -2660,18 +2662,18 @@
         <v>64</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J20" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K20" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K20" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21" s="16" t="s">
         <v>46</v>
@@ -2680,7 +2682,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E21" s="16">
         <v>15.0</v>
@@ -2695,18 +2697,18 @@
         <v>64</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J21" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K21" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>46</v>
@@ -2715,13 +2717,13 @@
         <v>47</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E22" s="16">
         <v>225.0</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G22" s="17">
         <v>46243.0</v>
@@ -2730,13 +2732,13 @@
         <v>64</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J22" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K22" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K22" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="23">
@@ -2750,7 +2752,7 @@
         <v>47</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E23" s="16">
         <v>7000.0</v>
@@ -2765,18 +2767,18 @@
         <v>64</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J23" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K23" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>51</v>
@@ -2791,27 +2793,27 @@
         <v>761000.0</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G24" s="17">
         <v>46243.0</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J24" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K24" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K24" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>51</v>
@@ -2835,18 +2837,18 @@
         <v>64</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J25" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K25" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K25" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B26" s="16" t="s">
         <v>51</v>
@@ -2861,7 +2863,7 @@
         <v>20500.0</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G26" s="17">
         <v>46243.0</v>
@@ -2870,13 +2872,13 @@
         <v>64</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J26" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K26" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K26" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -2905,62 +2907,62 @@
         <v>64</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J27" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K27" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E28" s="16">
         <v>10000.0</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G28" s="17">
         <v>46243.0</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J28" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K28" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K28" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E29" s="16">
         <v>12.0</v>
@@ -2972,51 +2974,51 @@
         <v>46243.0</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J29" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K29" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K29" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="B30" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>34</v>
       </c>
       <c r="E30" s="16">
         <v>250.0</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G30" s="17">
         <v>46243.0</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J30" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K30" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K30" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -3024,13 +3026,13 @@
         <v>66</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E31" s="16">
         <v>10000.0</v>
@@ -3042,21 +3044,21 @@
         <v>46243.0</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J31" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K31" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K31" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>51</v>
@@ -3071,27 +3073,27 @@
         <v>873668.0</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G32" s="17">
         <v>46243.0</v>
       </c>
       <c r="H32" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J32" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K32" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K32" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B33" s="16" t="s">
         <v>51</v>
@@ -3112,21 +3114,21 @@
         <v>46243.0</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J33" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K33" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K33" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B34" s="16" t="s">
         <v>51</v>
@@ -3141,22 +3143,22 @@
         <v>28500.0</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G34" s="17">
         <v>46243.0</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I34" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J34" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K34" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K34" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -3182,68 +3184,68 @@
         <v>46243.0</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J35" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="K35" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K35" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E36" s="16">
         <v>3299.0</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G36" s="17">
         <v>46243.0</v>
       </c>
       <c r="H36" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J36" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F37" s="16" t="s">
         <v>59</v>
@@ -3252,51 +3254,51 @@
         <v>46243.0</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J37" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K37" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G38" s="17">
         <v>46243.0</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J38" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -3304,13 +3306,13 @@
         <v>66</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E39" s="16">
         <v>18500.0</v>
@@ -3322,68 +3324,68 @@
         <v>46243.0</v>
       </c>
       <c r="H39" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J39" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B40" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G40" s="17">
         <v>46243.0</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J40" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F41" s="16" t="s">
         <v>59</v>
@@ -3392,51 +3394,51 @@
         <v>46243.0</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J41" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B42" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E42" s="16">
         <v>52.0</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G42" s="17">
         <v>46243.0</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J42" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -3447,10 +3449,10 @@
         <v>46</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E43" s="16">
         <v>3550.0</v>
@@ -3462,27 +3464,27 @@
         <v>46243.0</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I43" s="16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J43" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D44" s="16" t="s">
         <v>53</v>
@@ -3491,33 +3493,33 @@
         <v>107500.0</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G44" s="17">
         <v>46243.0</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I44" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J44" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K44" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>58</v>
-      </c>
-      <c r="B45" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>56</v>
       </c>
       <c r="D45" s="16" t="s">
         <v>53</v>
@@ -3532,21 +3534,21 @@
         <v>46243.0</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J45" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B46" s="16" t="s">
         <v>46</v>
@@ -3555,45 +3557,45 @@
         <v>47</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E46" s="16">
         <v>4000.0</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G46" s="17">
         <v>46243.0</v>
       </c>
       <c r="H46" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I46" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J46" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K46" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C47" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F47" s="16" t="s">
         <v>59</v>
@@ -3602,16 +3604,16 @@
         <v>46243.0</v>
       </c>
       <c r="H47" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I47" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J47" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K47" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -3619,13 +3621,13 @@
         <v>66</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E48" s="16">
         <v>205000.0</v>
@@ -3637,16 +3639,16 @@
         <v>46243.0</v>
       </c>
       <c r="H48" s="16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I48" s="16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J48" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K48" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -6482,20 +6484,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
+      <c r="A1" s="3" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>7</v>
@@ -6503,705 +6505,705 @@
     </row>
     <row r="4">
       <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="10"/>
     </row>
     <row r="5">
       <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="13" t="s">
-        <v>22</v>
+      <c r="B5" s="13"/>
+      <c r="C5" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="13" t="s">
-        <v>22</v>
+      <c r="B6" s="13"/>
+      <c r="C6" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>24</v>
+        <v>41</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13" t="s">
-        <v>22</v>
+      <c r="B7" s="13"/>
+      <c r="C7" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="13" t="s">
-        <v>22</v>
+      <c r="B8" s="13"/>
+      <c r="C8" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13" t="s">
-        <v>22</v>
+      <c r="B9" s="13"/>
+      <c r="C9" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13" t="s">
-        <v>22</v>
+      <c r="B10" s="13"/>
+      <c r="C10" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13" t="s">
-        <v>22</v>
+      <c r="B11" s="13"/>
+      <c r="C11" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>24</v>
+      <c r="E11" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13" t="s">
+      <c r="B12" s="13"/>
+      <c r="C12" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="13" t="s">
-        <v>34</v>
+      <c r="E12" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="13" t="s">
+      <c r="B13" s="13"/>
+      <c r="C13" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="13" t="s">
+      <c r="B14" s="13"/>
+      <c r="C14" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="13" t="s">
-        <v>34</v>
+      <c r="E14" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="13" t="s">
+      <c r="B15" s="13"/>
+      <c r="C15" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="13" t="s">
+      <c r="B16" s="13"/>
+      <c r="C16" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13" t="s">
-        <v>55</v>
+      <c r="B17" s="13"/>
+      <c r="C17" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E17" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
     </row>
     <row r="19">
       <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13" t="s">
-        <v>22</v>
+      <c r="B19" s="13"/>
+      <c r="C19" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="13" t="s">
-        <v>22</v>
+      <c r="B20" s="13"/>
+      <c r="C20" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>24</v>
+        <v>41</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13" t="s">
-        <v>22</v>
+      <c r="B21" s="13"/>
+      <c r="C21" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="13" t="s">
-        <v>22</v>
+      <c r="B22" s="13"/>
+      <c r="C22" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13" t="s">
-        <v>22</v>
+      <c r="B23" s="13"/>
+      <c r="C23" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="13" t="s">
-        <v>22</v>
+      <c r="B24" s="13"/>
+      <c r="C24" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13" t="s">
-        <v>22</v>
+      <c r="B25" s="13"/>
+      <c r="C25" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="13" t="s">
-        <v>24</v>
+      <c r="E25" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="13" t="s">
+      <c r="B26" s="13"/>
+      <c r="C26" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E26" s="13" t="s">
-        <v>34</v>
+      <c r="E26" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="11"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="13" t="s">
+      <c r="B27" s="13"/>
+      <c r="C27" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="11"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="13" t="s">
+      <c r="B28" s="13"/>
+      <c r="C28" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E28" s="13" t="s">
-        <v>34</v>
+      <c r="E28" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="13" t="s">
+      <c r="B29" s="13"/>
+      <c r="C29" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="13" t="s">
+      <c r="B30" s="13"/>
+      <c r="C30" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="13" t="s">
-        <v>55</v>
+      <c r="B31" s="13"/>
+      <c r="C31" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E31" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="7"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="10"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="11"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="13" t="s">
-        <v>22</v>
+      <c r="B33" s="13"/>
+      <c r="C33" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="13" t="s">
-        <v>22</v>
+      <c r="B34" s="13"/>
+      <c r="C34" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>24</v>
+        <v>41</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="11"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="13" t="s">
-        <v>22</v>
+      <c r="B35" s="13"/>
+      <c r="C35" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="11"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="13" t="s">
-        <v>22</v>
+      <c r="B36" s="13"/>
+      <c r="C36" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="11"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="13" t="s">
-        <v>22</v>
+      <c r="B37" s="13"/>
+      <c r="C37" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="11"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="13" t="s">
-        <v>22</v>
+      <c r="B38" s="13"/>
+      <c r="C38" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="11"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="13" t="s">
-        <v>22</v>
+      <c r="B39" s="13"/>
+      <c r="C39" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="13" t="s">
-        <v>24</v>
+      <c r="E39" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="11"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="13" t="s">
+      <c r="B40" s="13"/>
+      <c r="C40" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E40" s="13" t="s">
-        <v>34</v>
+      <c r="E40" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="11"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="13" t="s">
+      <c r="B41" s="13"/>
+      <c r="C41" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="11"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="13" t="s">
+      <c r="B42" s="13"/>
+      <c r="C42" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E42" s="13" t="s">
-        <v>34</v>
+      <c r="E42" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="13" t="s">
+      <c r="B43" s="13"/>
+      <c r="C43" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="11"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="13" t="s">
+      <c r="B44" s="13"/>
+      <c r="C44" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D44" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="E44" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="11"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="13" t="s">
-        <v>55</v>
+      <c r="B45" s="13"/>
+      <c r="C45" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E45" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="7"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="9"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="10"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="13" t="s">
-        <v>22</v>
+      <c r="B47" s="13"/>
+      <c r="C47" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="11"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="13" t="s">
-        <v>22</v>
+      <c r="B48" s="13"/>
+      <c r="C48" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E48" s="13" t="s">
-        <v>24</v>
+        <v>41</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="11"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="13" t="s">
-        <v>22</v>
+      <c r="B49" s="13"/>
+      <c r="C49" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="11"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="13" t="s">
-        <v>22</v>
+      <c r="B50" s="13"/>
+      <c r="C50" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E50" s="13" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="11"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="13" t="s">
-        <v>22</v>
+      <c r="B51" s="13"/>
+      <c r="C51" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E51" s="13" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="11"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="13" t="s">
-        <v>22</v>
+      <c r="B52" s="13"/>
+      <c r="C52" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="11"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="13" t="s">
-        <v>22</v>
+      <c r="B53" s="13"/>
+      <c r="C53" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="D53" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E53" s="13" t="s">
-        <v>24</v>
+      <c r="E53" s="14" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="11"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="13" t="s">
+      <c r="B54" s="13"/>
+      <c r="C54" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D54" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="13" t="s">
-        <v>34</v>
+      <c r="E54" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="11"/>
-      <c r="B55" s="12"/>
-      <c r="C55" s="13" t="s">
+      <c r="B55" s="13"/>
+      <c r="C55" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D55" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E55" s="13" t="s">
+      <c r="E55" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="11"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="13" t="s">
+      <c r="B56" s="13"/>
+      <c r="C56" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D56" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E56" s="13" t="s">
-        <v>34</v>
+      <c r="E56" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="11"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13" t="s">
+      <c r="B57" s="13"/>
+      <c r="C57" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D57" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="11"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="13" t="s">
+      <c r="B58" s="13"/>
+      <c r="C58" s="14" t="s">
         <v>51</v>
       </c>
       <c r="D58" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E58" s="13" t="s">
+      <c r="E58" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="11"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="13" t="s">
-        <v>55</v>
+      <c r="B59" s="13"/>
+      <c r="C59" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E59" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E59" s="14" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Notebook de analisis exploratorio + fix de duplicados en research manual
</commit_message>
<xml_diff>
--- a/data/manual/research_template_1.xlsx
+++ b/data/manual/research_template_1.xlsx
@@ -13,98 +13,98 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="141">
   <si>
     <t>LatamPulse — Template de Research Manual</t>
   </si>
   <si>
+    <t>country</t>
+  </si>
+  <si>
     <t>Checklist — 13 items x 4 países = 52 precios a investigar. Tildá acá a medida que cargás cada uno en la hoja 'Research'.</t>
   </si>
   <si>
     <t>Para qué sirve este archivo</t>
   </si>
   <si>
-    <t>country</t>
-  </si>
-  <si>
     <t>✓</t>
   </si>
   <si>
+    <t>Las fuentes oficiales (INDEC, IBGE, INE, DANE) no publican precios de items como Netflix, cine, cerveza en bar o Uber. Este template es donde cargás esos precios investigados a mano, con fecha y fuente — así el dato entra al pipeline con confidence = 'manual_research' y queda 100% trazable.</t>
+  </si>
+  <si>
+    <t>Cómo cargar cada fila</t>
+  </si>
+  <si>
+    <t>1. Andá a la hoja 'Research' (la pestaña de al lado).</t>
+  </si>
+  <si>
+    <t>2. La primera fila de datos (resaltada en amarillo) es un EJEMPLO — mostrá el formato esperado, no la borres, usala de referencia y agregá tus filas debajo.</t>
+  </si>
+  <si>
+    <t>3. Completá SOLO las columnas con fondo verde. El resto (usd_nominal, usd_ppp) se calcula después en transform.py — dejalas vacías.</t>
+  </si>
+  <si>
     <t>category</t>
   </si>
   <si>
     <t>item_name</t>
   </si>
   <si>
+    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
+  </si>
+  <si>
     <t>unit</t>
   </si>
   <si>
     <t>price_local</t>
   </si>
   <si>
+    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
+  </si>
+  <si>
     <t>currency</t>
   </si>
   <si>
+    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
+  </si>
+  <si>
     <t>date_captured</t>
   </si>
   <si>
+    <t>item</t>
+  </si>
+  <si>
     <t>source</t>
   </si>
   <si>
+    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
+  </si>
+  <si>
     <t>notes</t>
   </si>
   <si>
     <t>confidence</t>
   </si>
   <si>
-    <t>item</t>
-  </si>
-  <si>
     <t>captured_by</t>
   </si>
   <si>
+    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
+  </si>
+  <si>
+    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
+  </si>
+  <si>
     <t>AR</t>
   </si>
   <si>
-    <t>Las fuentes oficiales (INDEC, IBGE, INE, DANE) no publican precios de items como Netflix, cine, cerveza en bar o Uber. Este template es donde cargás esos precios investigados a mano, con fecha y fuente — así el dato entra al pipeline con confidence = 'manual_research' y queda 100% trazable.</t>
-  </si>
-  <si>
-    <t>Cómo cargar cada fila</t>
-  </si>
-  <si>
-    <t>1. Andá a la hoja 'Research' (la pestaña de al lado).</t>
-  </si>
-  <si>
-    <t>2. La primera fila de datos (resaltada en amarillo) es un EJEMPLO — mostrá el formato esperado, no la borres, usala de referencia y agregá tus filas debajo.</t>
-  </si>
-  <si>
-    <t>3. Completá SOLO las columnas con fondo verde. El resto (usd_nominal, usd_ppp) se calcula después en transform.py — dejalas vacías.</t>
-  </si>
-  <si>
-    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
-  </si>
-  <si>
-    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
-  </si>
-  <si>
-    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
-  </si>
-  <si>
-    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
-  </si>
-  <si>
-    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
-  </si>
-  <si>
     <t>entretenimiento</t>
   </si>
   <si>
     <t>Netflix Estándar (mensual)</t>
   </si>
   <si>
-    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
-  </si>
-  <si>
     <t>suscripcion_mensual</t>
   </si>
   <si>
@@ -135,18 +135,18 @@
     <t>UYU</t>
   </si>
   <si>
+    <t>Spotify Individual (mensual)</t>
+  </si>
+  <si>
+    <t>Menú/plato principal, restaurante gama media (1 persona)</t>
+  </si>
+  <si>
+    <t>Cerveza nacional 0.5L, en bar/restaurante</t>
+  </si>
+  <si>
     <t>lifecinemas.com.uy/candy</t>
   </si>
   <si>
-    <t>Spotify Individual (mensual)</t>
-  </si>
-  <si>
-    <t>Menú/plato principal, restaurante gama media (1 persona)</t>
-  </si>
-  <si>
-    <t>Cerveza nacional 0.5L, en bar/restaurante</t>
-  </si>
-  <si>
     <t>Café con leche/cortado, en cafetería</t>
   </si>
   <si>
@@ -180,18 +180,18 @@
     <t>Alquiler 2 ambientes, zona no céntrica (mensual)</t>
   </si>
   <si>
+    <t>salud</t>
+  </si>
+  <si>
+    <t>Prepaga/plan de salud privado, plan básico individual (mensual)</t>
+  </si>
+  <si>
     <t>Precio de lista sin promo, verificado en el sitio oficial</t>
   </si>
   <si>
-    <t>salud</t>
-  </si>
-  <si>
     <t>BR</t>
   </si>
   <si>
-    <t>Prepaga/plan de salud privado, plan básico individual (mensual)</t>
-  </si>
-  <si>
     <t>BRL</t>
   </si>
   <si>
@@ -264,19 +264,10 @@
     <t>Rango original: $30.000-60.000 ARS. Valor = punto medio</t>
   </si>
   <si>
-    <t>Rango original: R$80-150. Valor = punto medio</t>
-  </si>
-  <si>
     <t>Smart Fit / Fiter Uruguay</t>
   </si>
   <si>
     <t>Planes de $1.390-1.790 UYU. Valor = punto medio</t>
-  </si>
-  <si>
-    <t>Rango muy amplio: $60.000-400.000 COP. Confirmar si es gimnasio popular</t>
-  </si>
-  <si>
-    <t>Rango original: $3.000-8.000 ARS para 2-4km, UberX. Valor = punto medio</t>
   </si>
   <si>
     <t>Rango original: R$10-20. Valor = punto medio</t>
@@ -468,20 +459,14 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <b/>
       <sz val="11.0"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
       <sz val="10.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -493,16 +478,22 @@
     <font>
       <b/>
       <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <i/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <sz val="10.0"/>
       <color theme="1"/>
@@ -607,36 +598,36 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -894,72 +885,72 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2"/>
+      <c r="A2" s="3"/>
     </row>
     <row r="3" ht="18.0" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>2</v>
+      <c r="A3" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" ht="96.75" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" ht="18.0" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" ht="18.0" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" ht="51.75" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" ht="42.75" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" ht="49.5" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" ht="64.5" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" ht="39.75" customHeight="1">
+      <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2"/>
-    </row>
-    <row r="6" ht="18.0" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" ht="18.0" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" ht="51.75" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" ht="42.75" customHeight="1">
-      <c r="A9" s="2" t="s">
+    <row r="13" ht="70.5" customHeight="1">
+      <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" ht="64.5" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" ht="39.75" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" ht="70.5" customHeight="1">
-      <c r="A13" s="2" t="s">
+    <row r="14">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="6" t="s">
+    <row r="16" ht="91.5" customHeight="1">
+      <c r="A16" s="3" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="16" ht="91.5" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1972,186 +1963,186 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="A1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="4" t="s">
-        <v>15</v>
+      <c r="E1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="9">
         <v>14999.0</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="13">
         <v>46243.0</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="B3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="9">
         <v>570.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="13">
         <v>46239.0</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <v>7.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="13">
         <v>46237.0</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="B5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="9">
         <v>17900.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="13">
         <v>46243.0</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
@@ -2186,7 +2177,7 @@
         <v>66</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>37</v>
@@ -2218,13 +2209,13 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>38</v>
@@ -2253,13 +2244,13 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>38</v>
@@ -2291,10 +2282,10 @@
         <v>36</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>38</v>
@@ -2326,10 +2317,10 @@
         <v>66</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>38</v>
@@ -2358,10 +2349,10 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>44</v>
@@ -2393,10 +2384,10 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>44</v>
@@ -2431,7 +2422,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
@@ -2466,7 +2457,7 @@
         <v>66</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>44</v>
@@ -2498,10 +2489,10 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>45</v>
@@ -2533,10 +2524,10 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>45</v>
@@ -2545,19 +2536,19 @@
         <v>30</v>
       </c>
       <c r="E17" s="16">
-        <v>115.0</v>
+        <v>1590.0</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="G17" s="17">
         <v>46243.0</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>34</v>
@@ -2568,28 +2559,28 @@
     </row>
     <row r="18">
       <c r="A18" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E18" s="16">
-        <v>1590.0</v>
+        <v>15.0</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G18" s="17">
         <v>46243.0</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="I18" s="16" t="s">
         <v>85</v>
@@ -2603,22 +2594,22 @@
     </row>
     <row r="19">
       <c r="A19" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E19" s="16">
-        <v>150000.0</v>
+        <v>225.0</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G19" s="17">
         <v>46243.0</v>
@@ -2638,7 +2629,7 @@
     </row>
     <row r="20">
       <c r="A20" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B20" s="16" t="s">
         <v>46</v>
@@ -2650,10 +2641,10 @@
         <v>38</v>
       </c>
       <c r="E20" s="16">
-        <v>5500.0</v>
+        <v>7000.0</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G20" s="17">
         <v>46243.0</v>
@@ -2671,33 +2662,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E21" s="16">
-        <v>15.0</v>
+        <v>761000.0</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G21" s="17">
         <v>46243.0</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>34</v>
@@ -2706,24 +2697,24 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E22" s="16">
-        <v>225.0</v>
+        <v>2000.0</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G22" s="17">
         <v>46243.0</v>
@@ -2732,7 +2723,7 @@
         <v>64</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>34</v>
@@ -2741,24 +2732,24 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E23" s="16">
-        <v>7000.0</v>
+        <v>20500.0</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G23" s="17">
         <v>46243.0</v>
@@ -2767,7 +2758,7 @@
         <v>64</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J23" s="16" t="s">
         <v>34</v>
@@ -2778,7 +2769,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>51</v>
@@ -2790,16 +2781,16 @@
         <v>53</v>
       </c>
       <c r="E24" s="16">
-        <v>761000.0</v>
+        <v>1325000.0</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G24" s="17">
         <v>46243.0</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="I24" s="16" t="s">
         <v>92</v>
@@ -2813,31 +2804,31 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E25" s="16">
-        <v>2000.0</v>
+        <v>10000.0</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G25" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H25" s="16" t="s">
-        <v>64</v>
+      <c r="H25" s="19" t="s">
+        <v>93</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>34</v>
@@ -2848,31 +2839,31 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E26" s="16">
-        <v>20500.0</v>
+        <v>12.0</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G26" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H26" s="16" t="s">
-        <v>64</v>
+      <c r="H26" s="19" t="s">
+        <v>95</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>34</v>
@@ -2883,31 +2874,31 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E27" s="16">
-        <v>1325000.0</v>
+        <v>250.0</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G27" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H27" s="16" t="s">
-        <v>64</v>
+      <c r="H27" s="19" t="s">
+        <v>97</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>34</v>
@@ -2918,13 +2909,13 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D28" s="16" t="s">
         <v>38</v>
@@ -2933,16 +2924,16 @@
         <v>10000.0</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G28" s="17">
         <v>46243.0</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>34</v>
@@ -2953,31 +2944,31 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E29" s="16">
-        <v>12.0</v>
+        <v>873668.0</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G29" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H29" s="19" t="s">
-        <v>98</v>
+      <c r="H29" s="16" t="s">
+        <v>101</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J29" s="16" t="s">
         <v>34</v>
@@ -2988,31 +2979,31 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E30" s="16">
-        <v>250.0</v>
+        <v>2000.0</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G30" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H30" s="19" t="s">
-        <v>100</v>
+      <c r="H30" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>34</v>
@@ -3023,31 +3014,31 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E31" s="16">
-        <v>10000.0</v>
+        <v>28500.0</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G31" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H31" s="19" t="s">
-        <v>102</v>
+      <c r="H31" s="16" t="s">
+        <v>105</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="J31" s="16" t="s">
         <v>34</v>
@@ -3058,7 +3049,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>51</v>
@@ -3070,19 +3061,19 @@
         <v>53</v>
       </c>
       <c r="E32" s="16">
-        <v>873668.0</v>
+        <v>1600000.0</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G32" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H32" s="16" t="s">
-        <v>104</v>
+      <c r="H32" s="19" t="s">
+        <v>107</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>34</v>
@@ -3093,563 +3084,497 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E33" s="16">
-        <v>2000.0</v>
+        <v>3299.0</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G33" s="17">
         <v>46243.0</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>35</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="E34" s="16">
-        <v>28500.0</v>
+        <v>30</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>112</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G34" s="17">
         <v>46243.0</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I34" s="16" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="J34" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>35</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="E35" s="16">
-        <v>1600000.0</v>
+        <v>30</v>
+      </c>
+      <c r="E35" s="16" t="s">
+        <v>115</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="G35" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H35" s="19" t="s">
-        <v>110</v>
+      <c r="H35" s="16" t="s">
+        <v>116</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="J35" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>35</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D36" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E36" s="16">
-        <v>3299.0</v>
+        <v>18500.0</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G36" s="17">
         <v>46243.0</v>
       </c>
       <c r="H36" s="16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="J36" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G37" s="17">
         <v>46243.0</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="J37" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K37" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="G38" s="17">
         <v>46243.0</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="J38" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E39" s="16">
-        <v>18500.0</v>
+        <v>52.0</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G39" s="17">
         <v>46243.0</v>
       </c>
       <c r="H39" s="16" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="J39" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="16" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B40" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D40" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E40" s="16" t="s">
-        <v>123</v>
+      <c r="E40" s="16">
+        <v>3550.0</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="G40" s="17">
         <v>46243.0</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J40" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="16" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E41" s="16" t="s">
-        <v>126</v>
+        <v>53</v>
+      </c>
+      <c r="E41" s="16">
+        <v>107500.0</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G41" s="17">
         <v>46243.0</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="J41" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E42" s="16">
-        <v>52.0</v>
+        <v>310.0</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G42" s="17">
         <v>46243.0</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J42" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="16" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="B43" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="D43" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E43" s="16">
-        <v>3550.0</v>
+        <v>4000.0</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="G43" s="17">
         <v>46243.0</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I43" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="J43" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="16" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="E44" s="16">
-        <v>107500.0</v>
+        <v>30</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G44" s="17">
         <v>46243.0</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="I44" s="16" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J44" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K44" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="16" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E45" s="16">
-        <v>310.0</v>
+        <v>205000.0</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="G45" s="17">
         <v>46243.0</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="J45" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D46" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E46" s="16">
-        <v>4000.0</v>
-      </c>
-      <c r="F46" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="G46" s="17">
-        <v>46243.0</v>
-      </c>
-      <c r="H46" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="I46" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="J46" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="K46" s="16" t="s">
-        <v>114</v>
-      </c>
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
+      <c r="I46" s="20"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B47" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D47" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E47" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="G47" s="17">
-        <v>46243.0</v>
-      </c>
-      <c r="H47" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="I47" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="J47" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="K47" s="16" t="s">
-        <v>114</v>
-      </c>
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
+      <c r="I47" s="20"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="B48" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E48" s="16">
-        <v>205000.0</v>
-      </c>
-      <c r="F48" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="G48" s="17">
-        <v>46243.0</v>
-      </c>
-      <c r="H48" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="I48" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="J48" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="K48" s="16" t="s">
-        <v>114</v>
-      </c>
+      <c r="A48" s="20"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
+      <c r="H48" s="20"/>
+      <c r="I48" s="20"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="20"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="20"/>
@@ -5601,45 +5526,9 @@
       <c r="J198" s="20"/>
       <c r="K198" s="20"/>
     </row>
-    <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="20"/>
-      <c r="B199" s="20"/>
-      <c r="C199" s="20"/>
-      <c r="D199" s="20"/>
-      <c r="E199" s="20"/>
-      <c r="F199" s="20"/>
-      <c r="G199" s="20"/>
-      <c r="H199" s="20"/>
-      <c r="I199" s="20"/>
-      <c r="J199" s="20"/>
-      <c r="K199" s="20"/>
-    </row>
-    <row r="200" ht="15.75" customHeight="1">
-      <c r="A200" s="20"/>
-      <c r="B200" s="20"/>
-      <c r="C200" s="20"/>
-      <c r="D200" s="20"/>
-      <c r="E200" s="20"/>
-      <c r="F200" s="20"/>
-      <c r="G200" s="20"/>
-      <c r="H200" s="20"/>
-      <c r="I200" s="20"/>
-      <c r="J200" s="20"/>
-      <c r="K200" s="20"/>
-    </row>
-    <row r="201" ht="15.75" customHeight="1">
-      <c r="A201" s="20"/>
-      <c r="B201" s="20"/>
-      <c r="C201" s="20"/>
-      <c r="D201" s="20"/>
-      <c r="E201" s="20"/>
-      <c r="F201" s="20"/>
-      <c r="G201" s="20"/>
-      <c r="H201" s="20"/>
-      <c r="I201" s="20"/>
-      <c r="J201" s="20"/>
-      <c r="K201" s="20"/>
-    </row>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
     <row r="202" ht="15.75" customHeight="1"/>
     <row r="203" ht="15.75" customHeight="1"/>
     <row r="204" ht="15.75" customHeight="1"/>
@@ -6435,32 +6324,29 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Categoría inválida - Elegí una categoría de la lista — tiene que matchear el schema de prices." sqref="B2:B201">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Categoría inválida - Elegí una categoría de la lista — tiene que matchear el schema de prices." sqref="B2:B198">
       <formula1>"canasta_basica,vivienda,transporte,servicios,salud,entretenimiento"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J2:J201">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J198">
       <formula1>"manual_research"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="País inválido - Usá el código ISO2: AR, BR, UY o CO." sqref="A2:A201">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="País inválido - Usá el código ISO2: AR, BR, UY o CO." sqref="A2:A198">
       <formula1>"AR,BR,UY,CO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F201">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F198">
       <formula1>"ARS,BRL,UYU,COP,USD"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H3"/>
     <hyperlink r:id="rId2" ref="H4"/>
-    <hyperlink r:id="rId3" ref="H28"/>
-    <hyperlink r:id="rId4" ref="H29"/>
-    <hyperlink r:id="rId5" ref="H30"/>
-    <hyperlink r:id="rId6" ref="H31"/>
-    <hyperlink r:id="rId7" ref="H35"/>
+    <hyperlink r:id="rId3" ref="H25"/>
+    <hyperlink r:id="rId4" ref="H26"/>
+    <hyperlink r:id="rId5" ref="H27"/>
+    <hyperlink r:id="rId6" ref="H28"/>
+    <hyperlink r:id="rId7" ref="H32"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -6484,40 +6370,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>1</v>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>7</v>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5">
       <c r="A5" s="11"/>
-      <c r="B5" s="13"/>
+      <c r="B5" s="12"/>
       <c r="C5" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>30</v>
@@ -6525,12 +6411,12 @@
     </row>
     <row r="6">
       <c r="A6" s="11"/>
-      <c r="B6" s="13"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>30</v>
@@ -6538,9 +6424,9 @@
     </row>
     <row r="7">
       <c r="A7" s="11"/>
-      <c r="B7" s="13"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>37</v>
@@ -6551,12 +6437,12 @@
     </row>
     <row r="8">
       <c r="A8" s="11"/>
-      <c r="B8" s="13"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>38</v>
@@ -6564,12 +6450,12 @@
     </row>
     <row r="9">
       <c r="A9" s="11"/>
-      <c r="B9" s="13"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>38</v>
@@ -6577,9 +6463,9 @@
     </row>
     <row r="10">
       <c r="A10" s="11"/>
-      <c r="B10" s="13"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>44</v>
@@ -6590,9 +6476,9 @@
     </row>
     <row r="11">
       <c r="A11" s="11"/>
-      <c r="B11" s="13"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>45</v>
@@ -6603,7 +6489,7 @@
     </row>
     <row r="12">
       <c r="A12" s="11"/>
-      <c r="B12" s="13"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="14" t="s">
         <v>46</v>
       </c>
@@ -6616,7 +6502,7 @@
     </row>
     <row r="13">
       <c r="A13" s="11"/>
-      <c r="B13" s="13"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="14" t="s">
         <v>46</v>
       </c>
@@ -6629,7 +6515,7 @@
     </row>
     <row r="14">
       <c r="A14" s="11"/>
-      <c r="B14" s="13"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="14" t="s">
         <v>46</v>
       </c>
@@ -6642,7 +6528,7 @@
     </row>
     <row r="15">
       <c r="A15" s="11"/>
-      <c r="B15" s="13"/>
+      <c r="B15" s="12"/>
       <c r="C15" s="14" t="s">
         <v>51</v>
       </c>
@@ -6655,7 +6541,7 @@
     </row>
     <row r="16">
       <c r="A16" s="11"/>
-      <c r="B16" s="13"/>
+      <c r="B16" s="12"/>
       <c r="C16" s="14" t="s">
         <v>51</v>
       </c>
@@ -6668,12 +6554,12 @@
     </row>
     <row r="17">
       <c r="A17" s="11"/>
-      <c r="B17" s="13"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>58</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>53</v>
@@ -6681,19 +6567,19 @@
     </row>
     <row r="18">
       <c r="A18" s="7"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
       <c r="E18" s="10"/>
     </row>
     <row r="19">
       <c r="A19" s="11"/>
-      <c r="B19" s="13"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>30</v>
@@ -6701,12 +6587,12 @@
     </row>
     <row r="20">
       <c r="A20" s="11"/>
-      <c r="B20" s="13"/>
+      <c r="B20" s="12"/>
       <c r="C20" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>30</v>
@@ -6714,9 +6600,9 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="11"/>
-      <c r="B21" s="13"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>37</v>
@@ -6727,12 +6613,12 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="11"/>
-      <c r="B22" s="13"/>
+      <c r="B22" s="12"/>
       <c r="C22" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>38</v>
@@ -6740,12 +6626,12 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="11"/>
-      <c r="B23" s="13"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>38</v>
@@ -6753,9 +6639,9 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="11"/>
-      <c r="B24" s="13"/>
+      <c r="B24" s="12"/>
       <c r="C24" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>44</v>
@@ -6766,9 +6652,9 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="11"/>
-      <c r="B25" s="13"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>45</v>
@@ -6779,7 +6665,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="11"/>
-      <c r="B26" s="13"/>
+      <c r="B26" s="12"/>
       <c r="C26" s="14" t="s">
         <v>46</v>
       </c>
@@ -6792,7 +6678,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="11"/>
-      <c r="B27" s="13"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="14" t="s">
         <v>46</v>
       </c>
@@ -6805,7 +6691,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="11"/>
-      <c r="B28" s="13"/>
+      <c r="B28" s="12"/>
       <c r="C28" s="14" t="s">
         <v>46</v>
       </c>
@@ -6818,7 +6704,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="11"/>
-      <c r="B29" s="13"/>
+      <c r="B29" s="12"/>
       <c r="C29" s="14" t="s">
         <v>51</v>
       </c>
@@ -6831,7 +6717,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="11"/>
-      <c r="B30" s="13"/>
+      <c r="B30" s="12"/>
       <c r="C30" s="14" t="s">
         <v>51</v>
       </c>
@@ -6844,12 +6730,12 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="11"/>
-      <c r="B31" s="13"/>
+      <c r="B31" s="12"/>
       <c r="C31" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>58</v>
       </c>
       <c r="E31" s="14" t="s">
         <v>53</v>
@@ -6857,19 +6743,19 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="7"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
       <c r="E32" s="10"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="11"/>
-      <c r="B33" s="13"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>30</v>
@@ -6877,12 +6763,12 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="11"/>
-      <c r="B34" s="13"/>
+      <c r="B34" s="12"/>
       <c r="C34" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>30</v>
@@ -6890,9 +6776,9 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="11"/>
-      <c r="B35" s="13"/>
+      <c r="B35" s="12"/>
       <c r="C35" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>37</v>
@@ -6903,12 +6789,12 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="11"/>
-      <c r="B36" s="13"/>
+      <c r="B36" s="12"/>
       <c r="C36" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>38</v>
@@ -6916,12 +6802,12 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="11"/>
-      <c r="B37" s="13"/>
+      <c r="B37" s="12"/>
       <c r="C37" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>38</v>
@@ -6929,9 +6815,9 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="11"/>
-      <c r="B38" s="13"/>
+      <c r="B38" s="12"/>
       <c r="C38" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D38" s="11" t="s">
         <v>44</v>
@@ -6942,9 +6828,9 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="11"/>
-      <c r="B39" s="13"/>
+      <c r="B39" s="12"/>
       <c r="C39" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>45</v>
@@ -6955,7 +6841,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="11"/>
-      <c r="B40" s="13"/>
+      <c r="B40" s="12"/>
       <c r="C40" s="14" t="s">
         <v>46</v>
       </c>
@@ -6968,7 +6854,7 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="11"/>
-      <c r="B41" s="13"/>
+      <c r="B41" s="12"/>
       <c r="C41" s="14" t="s">
         <v>46</v>
       </c>
@@ -6981,7 +6867,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="11"/>
-      <c r="B42" s="13"/>
+      <c r="B42" s="12"/>
       <c r="C42" s="14" t="s">
         <v>46</v>
       </c>
@@ -6994,7 +6880,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="11"/>
-      <c r="B43" s="13"/>
+      <c r="B43" s="12"/>
       <c r="C43" s="14" t="s">
         <v>51</v>
       </c>
@@ -7007,7 +6893,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="11"/>
-      <c r="B44" s="13"/>
+      <c r="B44" s="12"/>
       <c r="C44" s="14" t="s">
         <v>51</v>
       </c>
@@ -7020,12 +6906,12 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="11"/>
-      <c r="B45" s="13"/>
+      <c r="B45" s="12"/>
       <c r="C45" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D45" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>58</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>53</v>
@@ -7033,19 +6919,19 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="7"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
       <c r="E46" s="10"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="11"/>
-      <c r="B47" s="13"/>
+      <c r="B47" s="12"/>
       <c r="C47" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E47" s="14" t="s">
         <v>30</v>
@@ -7053,12 +6939,12 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="11"/>
-      <c r="B48" s="13"/>
+      <c r="B48" s="12"/>
       <c r="C48" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>30</v>
@@ -7066,9 +6952,9 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="11"/>
-      <c r="B49" s="13"/>
+      <c r="B49" s="12"/>
       <c r="C49" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D49" s="11" t="s">
         <v>37</v>
@@ -7079,12 +6965,12 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="11"/>
-      <c r="B50" s="13"/>
+      <c r="B50" s="12"/>
       <c r="C50" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>38</v>
@@ -7092,12 +6978,12 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="11"/>
-      <c r="B51" s="13"/>
+      <c r="B51" s="12"/>
       <c r="C51" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>38</v>
@@ -7105,9 +6991,9 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="11"/>
-      <c r="B52" s="13"/>
+      <c r="B52" s="12"/>
       <c r="C52" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D52" s="11" t="s">
         <v>44</v>
@@ -7118,9 +7004,9 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="11"/>
-      <c r="B53" s="13"/>
+      <c r="B53" s="12"/>
       <c r="C53" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D53" s="11" t="s">
         <v>45</v>
@@ -7131,7 +7017,7 @@
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="11"/>
-      <c r="B54" s="13"/>
+      <c r="B54" s="12"/>
       <c r="C54" s="14" t="s">
         <v>46</v>
       </c>
@@ -7144,7 +7030,7 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="11"/>
-      <c r="B55" s="13"/>
+      <c r="B55" s="12"/>
       <c r="C55" s="14" t="s">
         <v>46</v>
       </c>
@@ -7157,7 +7043,7 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="11"/>
-      <c r="B56" s="13"/>
+      <c r="B56" s="12"/>
       <c r="C56" s="14" t="s">
         <v>46</v>
       </c>
@@ -7170,7 +7056,7 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="11"/>
-      <c r="B57" s="13"/>
+      <c r="B57" s="12"/>
       <c r="C57" s="14" t="s">
         <v>51</v>
       </c>
@@ -7183,7 +7069,7 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="11"/>
-      <c r="B58" s="13"/>
+      <c r="B58" s="12"/>
       <c r="C58" s="14" t="s">
         <v>51</v>
       </c>
@@ -7196,12 +7082,12 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="11"/>
-      <c r="B59" s="13"/>
+      <c r="B59" s="12"/>
       <c r="C59" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D59" s="11" t="s">
-        <v>58</v>
       </c>
       <c r="E59" s="14" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Mejora de calidad de datos: 9 fuentes confirmadas, fix de bug USD en compute_usd_values
</commit_message>
<xml_diff>
--- a/data/manual/research_template_1.xlsx
+++ b/data/manual/research_template_1.xlsx
@@ -13,92 +13,92 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="151">
   <si>
     <t>LatamPulse — Template de Research Manual</t>
   </si>
   <si>
+    <t>Para qué sirve este archivo</t>
+  </si>
+  <si>
+    <t>Las fuentes oficiales (INDEC, IBGE, INE, DANE) no publican precios de items como Netflix, cine, cerveza en bar o Uber. Este template es donde cargás esos precios investigados a mano, con fecha y fuente — así el dato entra al pipeline con confidence = 'manual_research' y queda 100% trazable.</t>
+  </si>
+  <si>
+    <t>Cómo cargar cada fila</t>
+  </si>
+  <si>
+    <t>1. Andá a la hoja 'Research' (la pestaña de al lado).</t>
+  </si>
+  <si>
+    <t>2. La primera fila de datos (resaltada en amarillo) es un EJEMPLO — mostrá el formato esperado, no la borres, usala de referencia y agregá tus filas debajo.</t>
+  </si>
+  <si>
+    <t>3. Completá SOLO las columnas con fondo verde. El resto (usd_nominal, usd_ppp) se calcula después en transform.py — dejalas vacías.</t>
+  </si>
+  <si>
+    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
+  </si>
+  <si>
+    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
+  </si>
+  <si>
+    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
+  </si>
+  <si>
+    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
+  </si>
+  <si>
+    <t>Checklist — 13 items x 4 países = 52 precios a investigar. Tildá acá a medida que cargás cada uno en la hoja 'Research'.</t>
+  </si>
+  <si>
     <t>country</t>
   </si>
   <si>
-    <t>Checklist — 13 items x 4 países = 52 precios a investigar. Tildá acá a medida que cargás cada uno en la hoja 'Research'.</t>
-  </si>
-  <si>
-    <t>Para qué sirve este archivo</t>
+    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
+  </si>
+  <si>
+    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>item_name</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>price_local</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>date_captured</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
+    <t>captured_by</t>
   </si>
   <si>
     <t>✓</t>
   </si>
   <si>
-    <t>Las fuentes oficiales (INDEC, IBGE, INE, DANE) no publican precios de items como Netflix, cine, cerveza en bar o Uber. Este template es donde cargás esos precios investigados a mano, con fecha y fuente — así el dato entra al pipeline con confidence = 'manual_research' y queda 100% trazable.</t>
-  </si>
-  <si>
-    <t>Cómo cargar cada fila</t>
-  </si>
-  <si>
-    <t>1. Andá a la hoja 'Research' (la pestaña de al lado).</t>
-  </si>
-  <si>
-    <t>2. La primera fila de datos (resaltada en amarillo) es un EJEMPLO — mostrá el formato esperado, no la borres, usala de referencia y agregá tus filas debajo.</t>
-  </si>
-  <si>
-    <t>3. Completá SOLO las columnas con fondo verde. El resto (usd_nominal, usd_ppp) se calcula después en transform.py — dejalas vacías.</t>
-  </si>
-  <si>
-    <t>category</t>
-  </si>
-  <si>
-    <t>item_name</t>
-  </si>
-  <si>
-    <t>4. country, category y confidence tienen dropdown — no escribas texto libre ahí, elegí de la lista para que el parseo en Python no se rompa por un typo.</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>price_local</t>
-  </si>
-  <si>
-    <t>5. source: no pongas solo 'Google'. Poné la fuente concreta — nombre del sitio/app y, si es posible, el link. Ej: 'App Rappi, Buenos Aires, pedido de prueba' o 'Netflix.com/ar precios oficiales'.</t>
-  </si>
-  <si>
-    <t>currency</t>
-  </si>
-  <si>
-    <t>6. date_captured: la fecha en que VOS viste ese precio, no la fecha de hoy si estás cargando atrasado. Formato AAAA-MM-DD.</t>
-  </si>
-  <si>
-    <t>date_captured</t>
+    <t>AR</t>
   </si>
   <si>
     <t>item</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>7. Si un precio varía mucho según el lugar (ej. alquiler, restaurante), especificá el criterio en notes — ej. 'restaurante gama media, zona no céntrica' — así después no comparamos peras con manzanas entre países.</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>confidence</t>
-  </si>
-  <si>
-    <t>captured_by</t>
-  </si>
-  <si>
-    <t>Por qué no tiene fórmulas de conversión ya cargadas</t>
-  </si>
-  <si>
-    <t>A propósito. La conversión a USD nominal y USD PPP se hace en transform.py con el tipo de cambio y factor PPP del DÍA de la extracción, no del día en que vos cargaste el precio acá. Si lo calculáramos en Excel con una tasa fija, quedaría desactualizado apenas cambie el dólar.</t>
-  </si>
-  <si>
-    <t>AR</t>
-  </si>
-  <si>
     <t>entretenimiento</t>
   </si>
   <si>
@@ -135,6 +135,9 @@
     <t>UYU</t>
   </si>
   <si>
+    <t>lifecinemas.com.uy/candy</t>
+  </si>
+  <si>
     <t>Spotify Individual (mensual)</t>
   </si>
   <si>
@@ -144,9 +147,6 @@
     <t>Cerveza nacional 0.5L, en bar/restaurante</t>
   </si>
   <si>
-    <t>lifecinemas.com.uy/candy</t>
-  </si>
-  <si>
     <t>Café con leche/cortado, en cafetería</t>
   </si>
   <si>
@@ -207,36 +207,24 @@
     <t>Cinépolis 16400, Cinemark Hoyts 18400, Atlas 17000-21000. Valor = promedio de los 3</t>
   </si>
   <si>
+    <t>CO</t>
+  </si>
+  <si>
+    <t>COP</t>
+  </si>
+  <si>
     <t>Fuente sin confirmar — pedir a Juani</t>
   </si>
   <si>
-    <t>Rango original: R$27-60, más caro jue-dom. Valor = punto medio</t>
-  </si>
-  <si>
-    <t>CO</t>
-  </si>
-  <si>
-    <t>COP</t>
-  </si>
-  <si>
     <t>Rango original: $12.000-30.500 COP. Valor = punto medio</t>
   </si>
   <si>
-    <t>Rango original: $15.000-30.000 ARS por persona con bebida. Valor = punto medio</t>
-  </si>
-  <si>
     <t>preciosmundi.com/brasil/precio-restaurantes ; dondedormiren.com/cuanto-cuesta-comer-en-brasil</t>
   </si>
   <si>
     <t>Rango original: 40-80 BRL por persona (plato individual). Valor = punto medio</t>
   </si>
   <si>
-    <t>Dato original: 2.010 UYU para 2 personas / 3 platos. Dividido entre 2 para aproximar 1 persona</t>
-  </si>
-  <si>
-    <t>Rango original: $30.000-60.000 COP por plato fuerte. Valor = punto medio</t>
-  </si>
-  <si>
     <t>Encuesta Maxirest (250 puntos de venta, mayoritariamente AMBA), vía infonegocios.info</t>
   </si>
   <si>
@@ -255,15 +243,9 @@
     <t>OJO: dato en USD, no BRL, y de feb 2025 (más viejo que el resto)</t>
   </si>
   <si>
-    <t>Rango original: $170-230 UYU. Valor = punto medio. No se encontró fuente confiable, revisar</t>
-  </si>
-  <si>
     <t>OJO: dato en USD, no COP, y de feb 2025</t>
   </si>
   <si>
-    <t>Rango original: $30.000-60.000 ARS. Valor = punto medio</t>
-  </si>
-  <si>
     <t>Smart Fit / Fiter Uruguay</t>
   </si>
   <si>
@@ -285,15 +267,6 @@
     <t>Promedio específico CABA de $761.000</t>
   </si>
   <si>
-    <t>Dato específico de Florianópolis, no necesariamente representativo de ciudad grande</t>
-  </si>
-  <si>
-    <t>Rango original: $16.000-25.000 UYU (Montevideo). Valor = punto medio</t>
-  </si>
-  <si>
-    <t>Rango original: $850.000-1.800.000 COP. Valor = punto medio</t>
-  </si>
-  <si>
     <t>preciosmundi.com/argentina/precio-restaurantes</t>
   </si>
   <si>
@@ -436,6 +409,63 @@
   </si>
   <si>
     <t>OJO: Bodytech es una cadena de gama media/alta, no la opción más económica del mercado colombiano — es el plan más barato QUE ENCONTRÉ con fuente ("hora naranja", franja 11-16h y noche). Podría no ser representativo de "gimnasio popular" — revisar si hay una opción más económica tipo Smart Fit Colombia</t>
+  </si>
+  <si>
+    <t>quintoandar.com.br — promedio studios/kitnets Florianópolis</t>
+  </si>
+  <si>
+    <t>Promedio real de la plataforma, rango R$1.180-4.500</t>
+  </si>
+  <si>
+    <t>fincaraiz.com.co — promedio apartaestudios Bogotá</t>
+  </si>
+  <si>
+    <t>Promedio real de la plataforma, desde $850.000</t>
+  </si>
+  <si>
+    <t>infocasas.com.uy — rango Centro, Montevideo</t>
+  </si>
+  <si>
+    <t>Fuente cotiza directo en USD (común en real estate uruguayo). Rango US$439-1.032, valor = punto medio</t>
+  </si>
+  <si>
+    <t>41.61</t>
+  </si>
+  <si>
+    <t>blog.nubank.com.br, citando Ingresso.com (mar 2025)</t>
+  </si>
+  <si>
+    <t>Rango São Paulo, sesión de semana, entrada completa: R$33,06-50,16. Artículo de 2025, podría estar algo desactualizado</t>
+  </si>
+  <si>
+    <t>iprofesional.com — relevamiento de precios, Smart Fit Plan Smart (oct 2024)</t>
+  </si>
+  <si>
+    <t>Plan de 1 sola sede, el más económico de la cadena. Artículo de 2024, precio probablemente desactualizado por inflación — revisar si se puede actualizar</t>
+  </si>
+  <si>
+    <t>expatistan.com — actualizado feb 2026</t>
+  </si>
+  <si>
+    <t>Precio promedio, capuccino, Montevideo</t>
+  </si>
+  <si>
+    <t>preciosmundi.com/argentina/precio-restaurantes (jul 2026)</t>
+  </si>
+  <si>
+    <t>Dato original: $81.852 ARS para 2 personas, 3 platos, gama media. Dividido entre 2 para aproximar 1 persona</t>
+  </si>
+  <si>
+    <t>preciosmundi.com/colombia/precio-restaurantes (jul 2026)</t>
+  </si>
+  <si>
+    <t>Dato original: $119.807 COP para 2 personas, 3 platos. Dividido entre 2</t>
+  </si>
+  <si>
+    <t>preciosmundi.com/uruguay (jun 2026)</t>
+  </si>
+  <si>
+    <t>Dato original: $2.007 UYU para 2 personas, 3 platos. Dividido entre 2</t>
   </si>
 </sst>
 </file>
@@ -459,12 +489,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FF1F4E78"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -483,17 +507,23 @@
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
-      <color theme="1"/>
+      <sz val="11.0"/>
+      <color rgb="FF1F4E78"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <i/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font/>
     <font>
       <sz val="10.0"/>
       <color theme="1"/>
@@ -539,14 +569,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -598,41 +628,41 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -885,72 +915,72 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3"/>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" ht="18.0" customHeight="1">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="96.75" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2"/>
+    </row>
+    <row r="6" ht="18.0" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="96.75" customHeight="1">
-      <c r="A4" s="3" t="s">
+    <row r="7" ht="18.0" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" ht="51.75" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3"/>
-    </row>
-    <row r="6" ht="18.0" customHeight="1">
-      <c r="A6" s="4" t="s">
+    <row r="9" ht="42.75" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="18.0" customHeight="1">
-      <c r="A7" s="3" t="s">
+    <row r="10" ht="49.5" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="51.75" customHeight="1">
-      <c r="A8" s="3" t="s">
+    <row r="11" ht="64.5" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" ht="42.75" customHeight="1">
-      <c r="A9" s="3" t="s">
+    <row r="12" ht="39.75" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" ht="64.5" customHeight="1">
-      <c r="A11" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" ht="39.75" customHeight="1">
-      <c r="A12" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
     <row r="13" ht="70.5" customHeight="1">
-      <c r="A13" s="3" t="s">
-        <v>21</v>
+      <c r="A13" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3"/>
+      <c r="A14" s="2"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="4" t="s">
-        <v>25</v>
+      <c r="A15" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" ht="91.5" customHeight="1">
-      <c r="A16" s="3" t="s">
-        <v>26</v>
+      <c r="A16" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1963,183 +1993,183 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="D1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="F1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="H1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="9" t="s">
+      <c r="A2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="7">
         <v>14999.0</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="9">
         <v>46243.0</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="7">
         <v>570.0</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="9">
         <v>46239.0</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="7">
         <v>7.0</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="9">
         <v>46237.0</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="7">
         <v>17900.0</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="9">
         <v>46243.0</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>28</v>
@@ -2151,19 +2181,19 @@
         <v>38</v>
       </c>
       <c r="E6" s="16">
-        <v>44.0</v>
+        <v>21250.0</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G6" s="17">
         <v>46243.0</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J6" s="16" t="s">
         <v>34</v>
@@ -2174,31 +2204,31 @@
     </row>
     <row r="7">
       <c r="A7" s="16" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E7" s="16">
-        <v>21250.0</v>
+        <v>60.0</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="G7" s="17">
         <v>46243.0</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J7" s="16" t="s">
         <v>34</v>
@@ -2209,19 +2239,19 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="16">
-        <v>22500.0</v>
+        <v>3336.0</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>31</v>
@@ -2230,10 +2260,10 @@
         <v>46243.0</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>34</v>
@@ -2250,25 +2280,25 @@
         <v>28</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="16">
-        <v>60.0</v>
+      <c r="E9" s="18" t="s">
+        <v>72</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="G9" s="17">
         <v>46243.0</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="J9" s="16" t="s">
         <v>34</v>
@@ -2279,31 +2309,31 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B10" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="16">
-        <v>1005.0</v>
+      <c r="E10" s="18" t="s">
+        <v>72</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="G10" s="17">
         <v>46243.0</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>34</v>
@@ -2314,31 +2344,31 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E11" s="16">
-        <v>45000.0</v>
+        <v>1590.0</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G11" s="17">
         <v>46243.0</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="J11" s="16" t="s">
         <v>34</v>
@@ -2349,31 +2379,31 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E12" s="16">
-        <v>3336.0</v>
+        <v>15.0</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G12" s="17">
         <v>46243.0</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>34</v>
@@ -2384,31 +2414,31 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>76</v>
+      <c r="E13" s="16">
+        <v>225.0</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="G13" s="17">
         <v>46243.0</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>34</v>
@@ -2419,31 +2449,31 @@
     </row>
     <row r="14">
       <c r="A14" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E14" s="16">
-        <v>200.0</v>
+        <v>7000.0</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="G14" s="17">
         <v>46243.0</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>34</v>
@@ -2452,33 +2482,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="16" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>76</v>
+        <v>53</v>
+      </c>
+      <c r="E15" s="16">
+        <v>761000.0</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>77</v>
+        <v>31</v>
       </c>
       <c r="G15" s="17">
         <v>46243.0</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>34</v>
@@ -2487,21 +2517,21 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E16" s="16">
-        <v>45000.0</v>
+        <v>10000.0</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>31</v>
@@ -2509,11 +2539,11 @@
       <c r="G16" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H16" s="16" t="s">
-        <v>64</v>
+      <c r="H16" s="19" t="s">
+        <v>84</v>
       </c>
       <c r="I16" s="16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>34</v>
@@ -2522,33 +2552,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E17" s="16">
-        <v>1590.0</v>
+        <v>12.0</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="G17" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H17" s="16" t="s">
-        <v>83</v>
+      <c r="H17" s="19" t="s">
+        <v>86</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>34</v>
@@ -2557,33 +2587,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E18" s="16">
-        <v>15.0</v>
+        <v>250.0</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="G18" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H18" s="16" t="s">
-        <v>64</v>
+      <c r="H18" s="19" t="s">
+        <v>88</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="J18" s="16" t="s">
         <v>34</v>
@@ -2592,33 +2622,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E19" s="16">
-        <v>225.0</v>
+        <v>10000.0</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="G19" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H19" s="16" t="s">
-        <v>64</v>
+      <c r="H19" s="19" t="s">
+        <v>90</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>34</v>
@@ -2627,33 +2657,33 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="16" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E20" s="16">
-        <v>7000.0</v>
+        <v>873668.0</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="G20" s="17">
         <v>46243.0</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>34</v>
@@ -2664,31 +2694,31 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B21" s="16" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E21" s="16">
-        <v>761000.0</v>
+        <v>2000.0</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G21" s="17">
         <v>46243.0</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>34</v>
@@ -2699,31 +2729,31 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>51</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E22" s="16">
-        <v>2000.0</v>
+        <v>28500.0</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="G22" s="17">
         <v>46243.0</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>34</v>
@@ -2734,31 +2764,31 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>51</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E23" s="16">
-        <v>20500.0</v>
+        <v>1600000.0</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="G23" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H23" s="16" t="s">
-        <v>64</v>
+      <c r="H23" s="19" t="s">
+        <v>98</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="J23" s="16" t="s">
         <v>34</v>
@@ -2769,527 +2799,527 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="16" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E24" s="16">
-        <v>1325000.0</v>
+        <v>3299.0</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="G24" s="17">
         <v>46243.0</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K24" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E25" s="16">
-        <v>10000.0</v>
+        <v>30</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G25" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H25" s="19" t="s">
-        <v>93</v>
+      <c r="H25" s="16" t="s">
+        <v>104</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K25" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B26" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E26" s="16">
-        <v>12.0</v>
+        <v>30</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>106</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="G26" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H26" s="19" t="s">
-        <v>95</v>
+      <c r="H26" s="16" t="s">
+        <v>107</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K26" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B27" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E27" s="16">
-        <v>250.0</v>
+        <v>18500.0</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="G27" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H27" s="19" t="s">
-        <v>97</v>
+      <c r="H27" s="16" t="s">
+        <v>100</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K27" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="16" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="D28" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E28" s="16">
-        <v>10000.0</v>
+      <c r="E28" s="16" t="s">
+        <v>111</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="G28" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H28" s="19" t="s">
-        <v>99</v>
+      <c r="H28" s="16" t="s">
+        <v>112</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K28" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>54</v>
+        <v>110</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="E29" s="16">
-        <v>873668.0</v>
+        <v>38</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>114</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G29" s="17">
         <v>46243.0</v>
       </c>
       <c r="H29" s="16" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="J29" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>54</v>
+        <v>110</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E30" s="16">
-        <v>2000.0</v>
+        <v>52.0</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="G30" s="17">
         <v>46243.0</v>
       </c>
       <c r="H30" s="16" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K30" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="16" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>54</v>
+        <v>110</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E31" s="16">
-        <v>28500.0</v>
+        <v>3550.0</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="G31" s="17">
         <v>46243.0</v>
       </c>
       <c r="H31" s="16" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="J31" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="16" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D32" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E32" s="16">
-        <v>1600000.0</v>
+        <v>107500.0</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="G32" s="17">
         <v>46243.0</v>
       </c>
-      <c r="H32" s="19" t="s">
-        <v>107</v>
+      <c r="H32" s="16" t="s">
+        <v>121</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>35</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="E33" s="16">
-        <v>3299.0</v>
+        <v>310.0</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G33" s="17">
         <v>46243.0</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="16" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" s="16" t="s">
-        <v>112</v>
+        <v>38</v>
+      </c>
+      <c r="E34" s="16">
+        <v>4000.0</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G34" s="17">
         <v>46243.0</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="I34" s="16" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J34" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="16" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B35" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D35" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="G35" s="17">
         <v>46243.0</v>
       </c>
       <c r="H35" s="16" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="J35" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B36" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D36" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E36" s="16">
-        <v>18500.0</v>
+        <v>205000.0</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G36" s="17">
         <v>46243.0</v>
       </c>
       <c r="H36" s="16" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="J36" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="16" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>119</v>
+        <v>52</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E37" s="16" t="s">
-        <v>120</v>
+        <v>53</v>
+      </c>
+      <c r="E37" s="16">
+        <v>1911.0</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G37" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J37" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K37" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>119</v>
+        <v>52</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38" s="16" t="s">
-        <v>123</v>
+        <v>53</v>
+      </c>
+      <c r="E38" s="16">
+        <v>2028619.0</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G38" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="J38" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -3297,244 +3327,244 @@
         <v>36</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>119</v>
+        <v>52</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E39" s="16">
-        <v>52.0</v>
+        <v>736.0</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="G39" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H39" s="16" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="J39" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="16" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="D40" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E40" s="16">
-        <v>3550.0</v>
+      <c r="E40" s="16" t="s">
+        <v>138</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="G40" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J40" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E41" s="16">
-        <v>107500.0</v>
+        <v>33990.0</v>
       </c>
       <c r="F41" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G41" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J41" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E42" s="16">
-        <v>310.0</v>
+        <v>252.0</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="G42" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J42" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D43" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E43" s="16">
-        <v>4000.0</v>
+        <v>40926.0</v>
       </c>
       <c r="F43" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G43" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="I43" s="16" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J43" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B44" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E44" s="16" t="s">
-        <v>136</v>
+        <v>38</v>
+      </c>
+      <c r="E44" s="16">
+        <v>59904.0</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G44" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="I44" s="16" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="J44" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K44" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="16" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E45" s="16">
-        <v>205000.0</v>
+        <v>1004.0</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G45" s="17">
-        <v>46243.0</v>
+        <v>46248.0</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="J45" s="16" t="s">
         <v>34</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -5396,136 +5426,16 @@
       <c r="J188" s="20"/>
       <c r="K188" s="20"/>
     </row>
-    <row r="189" ht="15.75" customHeight="1">
-      <c r="A189" s="20"/>
-      <c r="B189" s="20"/>
-      <c r="C189" s="20"/>
-      <c r="D189" s="20"/>
-      <c r="E189" s="20"/>
-      <c r="F189" s="20"/>
-      <c r="G189" s="20"/>
-      <c r="H189" s="20"/>
-      <c r="I189" s="20"/>
-      <c r="J189" s="20"/>
-      <c r="K189" s="20"/>
-    </row>
-    <row r="190" ht="15.75" customHeight="1">
-      <c r="A190" s="20"/>
-      <c r="B190" s="20"/>
-      <c r="C190" s="20"/>
-      <c r="D190" s="20"/>
-      <c r="E190" s="20"/>
-      <c r="F190" s="20"/>
-      <c r="G190" s="20"/>
-      <c r="H190" s="20"/>
-      <c r="I190" s="20"/>
-      <c r="J190" s="20"/>
-      <c r="K190" s="20"/>
-    </row>
-    <row r="191" ht="15.75" customHeight="1">
-      <c r="A191" s="20"/>
-      <c r="B191" s="20"/>
-      <c r="C191" s="20"/>
-      <c r="D191" s="20"/>
-      <c r="E191" s="20"/>
-      <c r="F191" s="20"/>
-      <c r="G191" s="20"/>
-      <c r="H191" s="20"/>
-      <c r="I191" s="20"/>
-      <c r="J191" s="20"/>
-      <c r="K191" s="20"/>
-    </row>
-    <row r="192" ht="15.75" customHeight="1">
-      <c r="A192" s="20"/>
-      <c r="B192" s="20"/>
-      <c r="C192" s="20"/>
-      <c r="D192" s="20"/>
-      <c r="E192" s="20"/>
-      <c r="F192" s="20"/>
-      <c r="G192" s="20"/>
-      <c r="H192" s="20"/>
-      <c r="I192" s="20"/>
-      <c r="J192" s="20"/>
-      <c r="K192" s="20"/>
-    </row>
-    <row r="193" ht="15.75" customHeight="1">
-      <c r="A193" s="20"/>
-      <c r="B193" s="20"/>
-      <c r="C193" s="20"/>
-      <c r="D193" s="20"/>
-      <c r="E193" s="20"/>
-      <c r="F193" s="20"/>
-      <c r="G193" s="20"/>
-      <c r="H193" s="20"/>
-      <c r="I193" s="20"/>
-      <c r="J193" s="20"/>
-      <c r="K193" s="20"/>
-    </row>
-    <row r="194" ht="15.75" customHeight="1">
-      <c r="A194" s="20"/>
-      <c r="B194" s="20"/>
-      <c r="C194" s="20"/>
-      <c r="D194" s="20"/>
-      <c r="E194" s="20"/>
-      <c r="F194" s="20"/>
-      <c r="G194" s="20"/>
-      <c r="H194" s="20"/>
-      <c r="I194" s="20"/>
-      <c r="J194" s="20"/>
-      <c r="K194" s="20"/>
-    </row>
-    <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="20"/>
-      <c r="B195" s="20"/>
-      <c r="C195" s="20"/>
-      <c r="D195" s="20"/>
-      <c r="E195" s="20"/>
-      <c r="F195" s="20"/>
-      <c r="G195" s="20"/>
-      <c r="H195" s="20"/>
-      <c r="I195" s="20"/>
-      <c r="J195" s="20"/>
-      <c r="K195" s="20"/>
-    </row>
-    <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="20"/>
-      <c r="B196" s="20"/>
-      <c r="C196" s="20"/>
-      <c r="D196" s="20"/>
-      <c r="E196" s="20"/>
-      <c r="F196" s="20"/>
-      <c r="G196" s="20"/>
-      <c r="H196" s="20"/>
-      <c r="I196" s="20"/>
-      <c r="J196" s="20"/>
-      <c r="K196" s="20"/>
-    </row>
-    <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="20"/>
-      <c r="B197" s="20"/>
-      <c r="C197" s="20"/>
-      <c r="D197" s="20"/>
-      <c r="E197" s="20"/>
-      <c r="F197" s="20"/>
-      <c r="G197" s="20"/>
-      <c r="H197" s="20"/>
-      <c r="I197" s="20"/>
-      <c r="J197" s="20"/>
-      <c r="K197" s="20"/>
-    </row>
-    <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="20"/>
-      <c r="B198" s="20"/>
-      <c r="C198" s="20"/>
-      <c r="D198" s="20"/>
-      <c r="E198" s="20"/>
-      <c r="F198" s="20"/>
-      <c r="G198" s="20"/>
-      <c r="H198" s="20"/>
-      <c r="I198" s="20"/>
-      <c r="J198" s="20"/>
-      <c r="K198" s="20"/>
-    </row>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
     <row r="199" ht="15.75" customHeight="1"/>
     <row r="200" ht="15.75" customHeight="1"/>
     <row r="201" ht="15.75" customHeight="1"/>
@@ -6314,39 +6224,29 @@
     <row r="984" ht="15.75" customHeight="1"/>
     <row r="985" ht="15.75" customHeight="1"/>
     <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Categoría inválida - Elegí una categoría de la lista — tiene que matchear el schema de prices." sqref="B2:B198">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Categoría inválida - Elegí una categoría de la lista — tiene que matchear el schema de prices." sqref="B2:B188">
       <formula1>"canasta_basica,vivienda,transporte,servicios,salud,entretenimiento"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J2:J198">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J188">
       <formula1>"manual_research"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="País inválido - Usá el código ISO2: AR, BR, UY o CO." sqref="A2:A198">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="País inválido - Usá el código ISO2: AR, BR, UY o CO." sqref="A2:A188">
       <formula1>"AR,BR,UY,CO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F198">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F188">
       <formula1>"ARS,BRL,UYU,COP,USD"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H3"/>
     <hyperlink r:id="rId2" ref="H4"/>
-    <hyperlink r:id="rId3" ref="H25"/>
-    <hyperlink r:id="rId4" ref="H26"/>
-    <hyperlink r:id="rId5" ref="H27"/>
-    <hyperlink r:id="rId6" ref="H28"/>
-    <hyperlink r:id="rId7" ref="H32"/>
+    <hyperlink r:id="rId3" ref="H16"/>
+    <hyperlink r:id="rId4" ref="H17"/>
+    <hyperlink r:id="rId5" ref="H18"/>
+    <hyperlink r:id="rId6" ref="H19"/>
+    <hyperlink r:id="rId7" ref="H23"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -6370,39 +6270,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
+      <c r="A1" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="11"/>
     </row>
     <row r="5">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -6410,25 +6310,25 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="11" t="s">
-        <v>40</v>
+      <c r="D6" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>37</v>
       </c>
       <c r="E7" s="14" t="s">
@@ -6436,38 +6336,38 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="13"/>
       <c r="C8" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>41</v>
+      <c r="D8" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="13"/>
       <c r="C9" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>42</v>
+      <c r="D9" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="13"/>
       <c r="C10" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E10" s="14" t="s">
@@ -6475,12 +6375,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="13"/>
       <c r="C11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="12" t="s">
         <v>45</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -6488,12 +6388,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="12" t="s">
         <v>47</v>
       </c>
       <c r="E12" s="14" t="s">
@@ -6501,12 +6401,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="13"/>
       <c r="C13" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E13" s="14" t="s">
@@ -6514,12 +6414,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="12" t="s">
         <v>50</v>
       </c>
       <c r="E14" s="14" t="s">
@@ -6527,12 +6427,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="12" t="s">
         <v>52</v>
       </c>
       <c r="E15" s="14" t="s">
@@ -6540,12 +6440,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E16" s="14" t="s">
@@ -6553,12 +6453,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="12" t="s">
         <v>56</v>
       </c>
       <c r="E17" s="14" t="s">
@@ -6566,19 +6466,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="10"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="11"/>
     </row>
     <row r="19">
-      <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E19" s="14" t="s">
@@ -6586,25 +6486,25 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11"/>
-      <c r="B20" s="12"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="11" t="s">
-        <v>40</v>
+      <c r="D20" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="12" t="s">
         <v>37</v>
       </c>
       <c r="E21" s="14" t="s">
@@ -6612,38 +6512,38 @@
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
+      <c r="A22" s="12"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="11" t="s">
-        <v>41</v>
+      <c r="D22" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="11" t="s">
-        <v>42</v>
+      <c r="D23" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
+      <c r="A24" s="12"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E24" s="14" t="s">
@@ -6651,12 +6551,12 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
+      <c r="A25" s="12"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="12" t="s">
         <v>45</v>
       </c>
       <c r="E25" s="14" t="s">
@@ -6664,12 +6564,12 @@
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="12" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="14" t="s">
@@ -6677,12 +6577,12 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="11"/>
-      <c r="B27" s="12"/>
+      <c r="A27" s="12"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E27" s="14" t="s">
@@ -6690,12 +6590,12 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="11"/>
-      <c r="B28" s="12"/>
+      <c r="A28" s="12"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="12" t="s">
         <v>50</v>
       </c>
       <c r="E28" s="14" t="s">
@@ -6703,12 +6603,12 @@
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
+      <c r="A29" s="12"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="12" t="s">
         <v>52</v>
       </c>
       <c r="E29" s="14" t="s">
@@ -6716,12 +6616,12 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E30" s="14" t="s">
@@ -6729,12 +6629,12 @@
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="12" t="s">
         <v>56</v>
       </c>
       <c r="E31" s="14" t="s">
@@ -6742,19 +6642,19 @@
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="10"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="11"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="11"/>
-      <c r="B33" s="12"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E33" s="14" t="s">
@@ -6762,25 +6662,25 @@
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
+      <c r="A34" s="12"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D34" s="11" t="s">
-        <v>40</v>
+      <c r="D34" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="11"/>
-      <c r="B35" s="12"/>
+      <c r="A35" s="12"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="12" t="s">
         <v>37</v>
       </c>
       <c r="E35" s="14" t="s">
@@ -6788,38 +6688,38 @@
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="11"/>
-      <c r="B36" s="12"/>
+      <c r="A36" s="12"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D36" s="11" t="s">
-        <v>41</v>
+      <c r="D36" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="11"/>
-      <c r="B37" s="12"/>
+      <c r="A37" s="12"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D37" s="11" t="s">
-        <v>42</v>
+      <c r="D37" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="11"/>
-      <c r="B38" s="12"/>
+      <c r="A38" s="12"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="D38" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E38" s="14" t="s">
@@ -6827,12 +6727,12 @@
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="11"/>
-      <c r="B39" s="12"/>
+      <c r="A39" s="12"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="11" t="s">
+      <c r="D39" s="12" t="s">
         <v>45</v>
       </c>
       <c r="E39" s="14" t="s">
@@ -6840,12 +6740,12 @@
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="11"/>
-      <c r="B40" s="12"/>
+      <c r="A40" s="12"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="12" t="s">
         <v>47</v>
       </c>
       <c r="E40" s="14" t="s">
@@ -6853,12 +6753,12 @@
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12"/>
+      <c r="A41" s="12"/>
+      <c r="B41" s="13"/>
       <c r="C41" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E41" s="14" t="s">
@@ -6866,12 +6766,12 @@
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="11"/>
-      <c r="B42" s="12"/>
+      <c r="A42" s="12"/>
+      <c r="B42" s="13"/>
       <c r="C42" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="12" t="s">
         <v>50</v>
       </c>
       <c r="E42" s="14" t="s">
@@ -6879,12 +6779,12 @@
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
+      <c r="A43" s="12"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="12" t="s">
         <v>52</v>
       </c>
       <c r="E43" s="14" t="s">
@@ -6892,12 +6792,12 @@
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="11"/>
-      <c r="B44" s="12"/>
+      <c r="A44" s="12"/>
+      <c r="B44" s="13"/>
       <c r="C44" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E44" s="14" t="s">
@@ -6905,12 +6805,12 @@
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="11"/>
-      <c r="B45" s="12"/>
+      <c r="A45" s="12"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="12" t="s">
         <v>56</v>
       </c>
       <c r="E45" s="14" t="s">
@@ -6918,19 +6818,19 @@
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="10"/>
+      <c r="A46" s="8"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="11"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
+      <c r="A47" s="12"/>
+      <c r="B47" s="13"/>
       <c r="C47" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E47" s="14" t="s">
@@ -6938,25 +6838,25 @@
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="11"/>
-      <c r="B48" s="12"/>
+      <c r="A48" s="12"/>
+      <c r="B48" s="13"/>
       <c r="C48" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D48" s="11" t="s">
-        <v>40</v>
+      <c r="D48" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="11"/>
-      <c r="B49" s="12"/>
+      <c r="A49" s="12"/>
+      <c r="B49" s="13"/>
       <c r="C49" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D49" s="12" t="s">
         <v>37</v>
       </c>
       <c r="E49" s="14" t="s">
@@ -6964,38 +6864,38 @@
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="11"/>
-      <c r="B50" s="12"/>
+      <c r="A50" s="12"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D50" s="11" t="s">
-        <v>41</v>
+      <c r="D50" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="11"/>
-      <c r="B51" s="12"/>
+      <c r="A51" s="12"/>
+      <c r="B51" s="13"/>
       <c r="C51" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D51" s="11" t="s">
-        <v>42</v>
+      <c r="D51" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="11"/>
-      <c r="B52" s="12"/>
+      <c r="A52" s="12"/>
+      <c r="B52" s="13"/>
       <c r="C52" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E52" s="14" t="s">
@@ -7003,12 +6903,12 @@
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="11"/>
-      <c r="B53" s="12"/>
+      <c r="A53" s="12"/>
+      <c r="B53" s="13"/>
       <c r="C53" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D53" s="11" t="s">
+      <c r="D53" s="12" t="s">
         <v>45</v>
       </c>
       <c r="E53" s="14" t="s">
@@ -7016,12 +6916,12 @@
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="11"/>
-      <c r="B54" s="12"/>
+      <c r="A54" s="12"/>
+      <c r="B54" s="13"/>
       <c r="C54" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="12" t="s">
         <v>47</v>
       </c>
       <c r="E54" s="14" t="s">
@@ -7029,12 +6929,12 @@
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="11"/>
-      <c r="B55" s="12"/>
+      <c r="A55" s="12"/>
+      <c r="B55" s="13"/>
       <c r="C55" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D55" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E55" s="14" t="s">
@@ -7042,12 +6942,12 @@
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="11"/>
-      <c r="B56" s="12"/>
+      <c r="A56" s="12"/>
+      <c r="B56" s="13"/>
       <c r="C56" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="12" t="s">
         <v>50</v>
       </c>
       <c r="E56" s="14" t="s">
@@ -7055,12 +6955,12 @@
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="11"/>
-      <c r="B57" s="12"/>
+      <c r="A57" s="12"/>
+      <c r="B57" s="13"/>
       <c r="C57" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D57" s="12" t="s">
         <v>52</v>
       </c>
       <c r="E57" s="14" t="s">
@@ -7068,12 +6968,12 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="11"/>
-      <c r="B58" s="12"/>
+      <c r="A58" s="12"/>
+      <c r="B58" s="13"/>
       <c r="C58" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E58" s="14" t="s">
@@ -7081,12 +6981,12 @@
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="11"/>
-      <c r="B59" s="12"/>
+      <c r="A59" s="12"/>
+      <c r="B59" s="13"/>
       <c r="C59" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="12" t="s">
         <v>56</v>
       </c>
       <c r="E59" s="14" t="s">

</xml_diff>